<commit_message>
lưu code de lay ve lan cuoi
</commit_message>
<xml_diff>
--- a/auto_marketing_client/public/files/mau_campaign.xlsx
+++ b/auto_marketing_client/public/files/mau_campaign.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngock\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E28E49E3-69B8-4A78-B204-20DFBBC5B8CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1EE3772-C411-46A4-9164-6298FDED8058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="690" windowWidth="21600" windowHeight="11295" xr2:uid="{E7933397-5124-43DF-A199-47E25EC42A4A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E7933397-5124-43DF-A199-47E25EC42A4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,9 +30,6 @@
     <t>Tên chiến dịch</t>
   </si>
   <si>
-    <t xml:space="preserve">Chi tiết chiến dịch </t>
-  </si>
-  <si>
     <t xml:space="preserve">Ngày bắt đầu </t>
   </si>
   <si>
@@ -49,6 +46,9 @@
   </si>
   <si>
     <t>Chiến dịch B</t>
+  </si>
+  <si>
+    <t>Chi tiết</t>
   </si>
 </sst>
 </file>
@@ -105,9 +105,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -145,7 +145,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -251,7 +251,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -393,7 +393,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -402,34 +402,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A239F818-C87E-423B-9825-5C649A438B0C}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="33.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" customWidth="1"/>
-    <col min="3" max="3" width="12.140625" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="1" max="1" width="33.5546875" customWidth="1"/>
+    <col min="2" max="2" width="19.44140625" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
       </c>
       <c r="C2" s="1">
         <v>45888</v>
@@ -438,12 +438,12 @@
         <v>45890</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1">
         <v>45901</v>

</xml_diff>